<commit_message>
docs: adjust five year growth assumption
</commit_message>
<xml_diff>
--- a/deck-system/decks/umee-sbcs-kintone-plan-3980/exports/umee-kintonepack-5yr-revenue-plan.xlsx
+++ b/deck-system/decks/umee-sbcs-kintone-plan-3980/exports/umee-kintonepack-5yr-revenue-plan.xlsx
@@ -74,7 +74,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>既存Excelが切れるFY29Q2以降、Umee全体売上計画は四半期ごとに1.3倍成長として延長</t>
+          <t>既存Excelが切れるFY29Q2以降、Umee全体売上計画は四半期ごとに1.05倍成長として延長</t>
         </is>
       </c>
     </row>
@@ -626,31 +626,31 @@
         </is>
       </c>
       <c r="B14">
-        <v>8568</v>
+        <v>6921</v>
       </c>
       <c r="C14">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D14">
-        <v>2212</v>
+        <v>369</v>
       </c>
       <c r="E14">
-        <v>4734</v>
+        <v>2891</v>
       </c>
       <c r="F14">
-        <v>1106</v>
+        <v>184</v>
       </c>
       <c r="G14">
-        <v>2368</v>
+        <v>1446</v>
       </c>
       <c r="H14">
-        <v>474</v>
+        <v>289</v>
       </c>
       <c r="I14">
-        <v>2044</v>
+        <v>1410</v>
       </c>
       <c r="J14">
-        <v>9751</v>
+        <v>9117</v>
       </c>
     </row>
     <row r="15">
@@ -660,31 +660,31 @@
         </is>
       </c>
       <c r="B15">
-        <v>11139</v>
+        <v>7267</v>
       </c>
       <c r="C15">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D15">
-        <v>2875</v>
+        <v>387</v>
       </c>
       <c r="E15">
-        <v>7373</v>
+        <v>3042</v>
       </c>
       <c r="F15">
-        <v>1438</v>
+        <v>194</v>
       </c>
       <c r="G15">
-        <v>3688</v>
+        <v>1522</v>
       </c>
       <c r="H15">
-        <v>738</v>
+        <v>304</v>
       </c>
       <c r="I15">
-        <v>3001</v>
+        <v>1511</v>
       </c>
       <c r="J15">
-        <v>12752</v>
+        <v>10628</v>
       </c>
     </row>
     <row r="16">
@@ -694,31 +694,31 @@
         </is>
       </c>
       <c r="B16">
-        <v>14480</v>
+        <v>7630</v>
       </c>
       <c r="C16">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D16">
-        <v>3738</v>
+        <v>406</v>
       </c>
       <c r="E16">
-        <v>10828</v>
+        <v>3165</v>
       </c>
       <c r="F16">
-        <v>1869</v>
+        <v>203</v>
       </c>
       <c r="G16">
-        <v>5415</v>
+        <v>1583</v>
       </c>
       <c r="H16">
-        <v>1083</v>
+        <v>317</v>
       </c>
       <c r="I16">
-        <v>4248</v>
+        <v>1612</v>
       </c>
       <c r="J16">
-        <v>17000</v>
+        <v>12241</v>
       </c>
     </row>
     <row r="17">
@@ -728,31 +728,31 @@
         </is>
       </c>
       <c r="B17">
-        <v>18824</v>
+        <v>8011</v>
       </c>
       <c r="C17">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D17">
-        <v>4859</v>
+        <v>427</v>
       </c>
       <c r="E17">
-        <v>15380</v>
+        <v>3285</v>
       </c>
       <c r="F17">
-        <v>2430</v>
+        <v>214</v>
       </c>
       <c r="G17">
-        <v>7692</v>
+        <v>1644</v>
       </c>
       <c r="H17">
-        <v>1538</v>
+        <v>329</v>
       </c>
       <c r="I17">
-        <v>5877</v>
+        <v>1718</v>
       </c>
       <c r="J17">
-        <v>22877</v>
+        <v>13959</v>
       </c>
     </row>
     <row r="18">
@@ -762,31 +762,31 @@
         </is>
       </c>
       <c r="B18">
-        <v>24472</v>
+        <v>8412</v>
       </c>
       <c r="C18">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D18">
-        <v>6317</v>
+        <v>448</v>
       </c>
       <c r="E18">
-        <v>20516</v>
+        <v>3473</v>
       </c>
       <c r="F18">
-        <v>3158</v>
+        <v>224</v>
       </c>
       <c r="G18">
-        <v>10259</v>
+        <v>1738</v>
       </c>
       <c r="H18">
-        <v>2052</v>
+        <v>348</v>
       </c>
       <c r="I18">
-        <v>7999</v>
+        <v>1820</v>
       </c>
       <c r="J18">
-        <v>30876</v>
+        <v>15779</v>
       </c>
     </row>
     <row r="19">
@@ -796,31 +796,31 @@
         </is>
       </c>
       <c r="B19">
-        <v>31813</v>
+        <v>8833</v>
       </c>
       <c r="C19">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D19">
-        <v>8212</v>
+        <v>470</v>
       </c>
       <c r="E19">
-        <v>27215</v>
+        <v>3675</v>
       </c>
       <c r="F19">
-        <v>4106</v>
+        <v>235</v>
       </c>
       <c r="G19">
-        <v>13608</v>
+        <v>1838</v>
       </c>
       <c r="H19">
-        <v>2722</v>
+        <v>368</v>
       </c>
       <c r="I19">
-        <v>10774</v>
+        <v>1930</v>
       </c>
       <c r="J19">
-        <v>41651</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="20">
@@ -830,31 +830,31 @@
         </is>
       </c>
       <c r="B20">
-        <v>41357</v>
+        <v>9274</v>
       </c>
       <c r="C20">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D20">
-        <v>10676</v>
+        <v>494</v>
       </c>
       <c r="E20">
-        <v>35932</v>
+        <v>3875</v>
       </c>
       <c r="F20">
-        <v>5338</v>
+        <v>247</v>
       </c>
       <c r="G20">
-        <v>17967</v>
+        <v>1939</v>
       </c>
       <c r="H20">
-        <v>3593</v>
+        <v>388</v>
       </c>
       <c r="I20">
-        <v>14387</v>
+        <v>2038</v>
       </c>
       <c r="J20">
-        <v>56038</v>
+        <v>19748</v>
       </c>
     </row>
     <row r="21">
@@ -864,31 +864,31 @@
         </is>
       </c>
       <c r="B21">
-        <v>53764</v>
+        <v>9738</v>
       </c>
       <c r="C21">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D21">
-        <v>13878</v>
+        <v>519</v>
       </c>
       <c r="E21">
-        <v>47282</v>
+        <v>4083</v>
       </c>
       <c r="F21">
-        <v>6939</v>
+        <v>260</v>
       </c>
       <c r="G21">
-        <v>23642</v>
+        <v>2043</v>
       </c>
       <c r="H21">
-        <v>4728</v>
+        <v>409</v>
       </c>
       <c r="I21">
-        <v>19097</v>
+        <v>2150</v>
       </c>
       <c r="J21">
-        <v>75135</v>
+        <v>21898</v>
       </c>
     </row>
   </sheetData>
@@ -1028,19 +1028,19 @@
         </is>
       </c>
       <c r="C5">
-        <v>18824</v>
+        <v>8011</v>
       </c>
       <c r="D5">
-        <v>7692</v>
+        <v>1644</v>
       </c>
       <c r="E5">
-        <v>1538</v>
+        <v>329</v>
       </c>
       <c r="F5">
-        <v>15170</v>
+        <v>6252</v>
       </c>
       <c r="G5">
-        <v>22877</v>
+        <v>13959</v>
       </c>
     </row>
     <row r="6">
@@ -1055,19 +1055,19 @@
         </is>
       </c>
       <c r="C6">
-        <v>53764</v>
+        <v>9738</v>
       </c>
       <c r="D6">
-        <v>23642</v>
+        <v>2043</v>
       </c>
       <c r="E6">
-        <v>4728</v>
+        <v>409</v>
       </c>
       <c r="F6">
-        <v>52258</v>
+        <v>7939</v>
       </c>
       <c r="G6">
-        <v>75135</v>
+        <v>21898</v>
       </c>
     </row>
   </sheetData>
@@ -1546,31 +1546,31 @@
         </is>
       </c>
       <c r="B14">
-        <v>8568</v>
+        <v>6921</v>
       </c>
       <c r="C14">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D14">
-        <v>2212</v>
+        <v>369</v>
       </c>
       <c r="E14">
-        <v>4734</v>
+        <v>2891</v>
       </c>
       <c r="F14">
-        <v>1106</v>
+        <v>184</v>
       </c>
       <c r="G14">
-        <v>2368</v>
+        <v>1446</v>
       </c>
       <c r="H14">
-        <v>474</v>
+        <v>289</v>
       </c>
       <c r="I14">
-        <v>2452</v>
+        <v>1605</v>
       </c>
       <c r="J14">
-        <v>11696</v>
+        <v>10849</v>
       </c>
     </row>
     <row r="15">
@@ -1580,31 +1580,31 @@
         </is>
       </c>
       <c r="B15">
-        <v>11139</v>
+        <v>7267</v>
       </c>
       <c r="C15">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D15">
-        <v>2875</v>
+        <v>387</v>
       </c>
       <c r="E15">
-        <v>7373</v>
+        <v>3042</v>
       </c>
       <c r="F15">
-        <v>1438</v>
+        <v>194</v>
       </c>
       <c r="G15">
-        <v>3688</v>
+        <v>1522</v>
       </c>
       <c r="H15">
-        <v>738</v>
+        <v>304</v>
       </c>
       <c r="I15">
-        <v>3697</v>
+        <v>1708</v>
       </c>
       <c r="J15">
-        <v>15393</v>
+        <v>12557</v>
       </c>
     </row>
     <row r="16">
@@ -1614,31 +1614,31 @@
         </is>
       </c>
       <c r="B16">
-        <v>14480</v>
+        <v>7630</v>
       </c>
       <c r="C16">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D16">
-        <v>3738</v>
+        <v>406</v>
       </c>
       <c r="E16">
-        <v>10828</v>
+        <v>3165</v>
       </c>
       <c r="F16">
-        <v>1869</v>
+        <v>203</v>
       </c>
       <c r="G16">
-        <v>5415</v>
+        <v>1583</v>
       </c>
       <c r="H16">
-        <v>1083</v>
+        <v>317</v>
       </c>
       <c r="I16">
-        <v>5323</v>
+        <v>1803</v>
       </c>
       <c r="J16">
-        <v>20716</v>
+        <v>14360</v>
       </c>
     </row>
     <row r="17">
@@ -1648,31 +1648,31 @@
         </is>
       </c>
       <c r="B17">
-        <v>18824</v>
+        <v>8011</v>
       </c>
       <c r="C17">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D17">
-        <v>4859</v>
+        <v>427</v>
       </c>
       <c r="E17">
-        <v>15380</v>
+        <v>3285</v>
       </c>
       <c r="F17">
-        <v>2430</v>
+        <v>214</v>
       </c>
       <c r="G17">
-        <v>7692</v>
+        <v>1644</v>
       </c>
       <c r="H17">
-        <v>1538</v>
+        <v>329</v>
       </c>
       <c r="I17">
-        <v>7456</v>
+        <v>1901</v>
       </c>
       <c r="J17">
-        <v>28172</v>
+        <v>16262</v>
       </c>
     </row>
     <row r="18">
@@ -1682,31 +1682,31 @@
         </is>
       </c>
       <c r="B18">
-        <v>24472</v>
+        <v>8412</v>
       </c>
       <c r="C18">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D18">
-        <v>6317</v>
+        <v>448</v>
       </c>
       <c r="E18">
-        <v>20516</v>
+        <v>3473</v>
       </c>
       <c r="F18">
-        <v>3158</v>
+        <v>224</v>
       </c>
       <c r="G18">
-        <v>10259</v>
+        <v>1738</v>
       </c>
       <c r="H18">
-        <v>2052</v>
+        <v>348</v>
       </c>
       <c r="I18">
-        <v>10052</v>
+        <v>2013</v>
       </c>
       <c r="J18">
-        <v>38224</v>
+        <v>18275</v>
       </c>
     </row>
     <row r="19">
@@ -1716,31 +1716,31 @@
         </is>
       </c>
       <c r="B19">
-        <v>31813</v>
+        <v>8833</v>
       </c>
       <c r="C19">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D19">
-        <v>8212</v>
+        <v>470</v>
       </c>
       <c r="E19">
-        <v>27215</v>
+        <v>3675</v>
       </c>
       <c r="F19">
-        <v>4106</v>
+        <v>235</v>
       </c>
       <c r="G19">
-        <v>13608</v>
+        <v>1838</v>
       </c>
       <c r="H19">
-        <v>2722</v>
+        <v>368</v>
       </c>
       <c r="I19">
-        <v>13443</v>
+        <v>2133</v>
       </c>
       <c r="J19">
-        <v>51667</v>
+        <v>20407</v>
       </c>
     </row>
     <row r="20">
@@ -1750,31 +1750,31 @@
         </is>
       </c>
       <c r="B20">
-        <v>41357</v>
+        <v>9274</v>
       </c>
       <c r="C20">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D20">
-        <v>10676</v>
+        <v>494</v>
       </c>
       <c r="E20">
-        <v>35932</v>
+        <v>3875</v>
       </c>
       <c r="F20">
-        <v>5338</v>
+        <v>247</v>
       </c>
       <c r="G20">
-        <v>17967</v>
+        <v>1939</v>
       </c>
       <c r="H20">
-        <v>3593</v>
+        <v>388</v>
       </c>
       <c r="I20">
-        <v>17856</v>
+        <v>2251</v>
       </c>
       <c r="J20">
-        <v>69523</v>
+        <v>22658</v>
       </c>
     </row>
     <row r="21">
@@ -1784,31 +1784,31 @@
         </is>
       </c>
       <c r="B21">
-        <v>53764</v>
+        <v>9738</v>
       </c>
       <c r="C21">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="D21">
-        <v>13878</v>
+        <v>519</v>
       </c>
       <c r="E21">
-        <v>47282</v>
+        <v>4083</v>
       </c>
       <c r="F21">
-        <v>6939</v>
+        <v>260</v>
       </c>
       <c r="G21">
-        <v>23642</v>
+        <v>2043</v>
       </c>
       <c r="H21">
-        <v>4728</v>
+        <v>409</v>
       </c>
       <c r="I21">
-        <v>23606</v>
+        <v>2373</v>
       </c>
       <c r="J21">
-        <v>93129</v>
+        <v>25031</v>
       </c>
     </row>
   </sheetData>
@@ -1948,19 +1948,19 @@
         </is>
       </c>
       <c r="C5">
-        <v>18824</v>
+        <v>8011</v>
       </c>
       <c r="D5">
-        <v>7692</v>
+        <v>1644</v>
       </c>
       <c r="E5">
-        <v>1538</v>
+        <v>329</v>
       </c>
       <c r="F5">
-        <v>18928</v>
+        <v>7017</v>
       </c>
       <c r="G5">
-        <v>28172</v>
+        <v>16262</v>
       </c>
     </row>
     <row r="6">
@@ -1975,19 +1975,19 @@
         </is>
       </c>
       <c r="C6">
-        <v>53764</v>
+        <v>9738</v>
       </c>
       <c r="D6">
-        <v>23642</v>
+        <v>2043</v>
       </c>
       <c r="E6">
-        <v>4728</v>
+        <v>409</v>
       </c>
       <c r="F6">
-        <v>64957</v>
+        <v>8769</v>
       </c>
       <c r="G6">
-        <v>93129</v>
+        <v>25031</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: reflect updated fy29 revenue values
</commit_message>
<xml_diff>
--- a/deck-system/decks/umee-sbcs-kintone-plan-3980/exports/umee-kintonepack-5yr-revenue-plan.xlsx
+++ b/deck-system/decks/umee-sbcs-kintone-plan-3980/exports/umee-kintonepack-5yr-revenue-plan.xlsx
@@ -69,82 +69,94 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5か年延長</t>
+          <t>追加提示値</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>既存Excelが切れるFY29Q2以降、Umee全体売上計画は四半期ごとに1.05倍成長として延長</t>
+          <t>FY29Q3は70,304、FY29Q4は74,698を反映</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SBC&amp;S取扱見込</t>
+          <t>5か年延長</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Umee Tier3計画IDの50%</t>
+          <t>FY30Q1以降、Umee全体売上計画は四半期ごとに1.05倍成長として延長</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>契約法人</t>
+          <t>SBC&amp;S取扱見込</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SBC&amp;S積上ID ÷ 5ID/法人</t>
+          <t>Umee Tier3計画IDの50%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>継続率</t>
+          <t>契約法人</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>契約開始1年後50%、以降1年ごとに80%</t>
+          <t>SBC&amp;S積上ID ÷ 5ID/法人</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>貴社支払いレベニュー額</t>
+          <t>継続率</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kintone Pack販売価格 ÷ 1.3 × 稼働SBC&amp;S ID × 3ヶ月</t>
+          <t>契約開始1年後50%、以降1年ごとに80%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>価格パターン</t>
+          <t>貴社支払いレベニュー額</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>初年度2,980円または3,980円 / ID / 月、2年目以降5,980円 / ID / 月</t>
+          <t>Kintone Pack販売価格 ÷ 1.3 × 稼働SBC&amp;S ID × 3ヶ月</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>価格パターン</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>初年度2,980円または3,980円 / ID / 月、2年目以降5,980円 / ID / 月</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>FrontAX</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>本試算には含めない</t>
         </is>
@@ -626,31 +638,31 @@
         </is>
       </c>
       <c r="B14">
-        <v>6921</v>
+        <v>7030</v>
       </c>
       <c r="C14">
-        <v>1.05</v>
+        <v>1.067</v>
       </c>
       <c r="D14">
-        <v>369</v>
+        <v>491</v>
       </c>
       <c r="E14">
-        <v>2891</v>
+        <v>3013</v>
       </c>
       <c r="F14">
-        <v>184</v>
+        <v>246</v>
       </c>
       <c r="G14">
-        <v>1446</v>
+        <v>1508</v>
       </c>
       <c r="H14">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="I14">
-        <v>1410</v>
+        <v>1452</v>
       </c>
       <c r="J14">
-        <v>9117</v>
+        <v>9160</v>
       </c>
     </row>
     <row r="15">
@@ -660,31 +672,31 @@
         </is>
       </c>
       <c r="B15">
-        <v>7267</v>
+        <v>7470</v>
       </c>
       <c r="C15">
-        <v>1.05</v>
+        <v>1.062</v>
       </c>
       <c r="D15">
-        <v>387</v>
+        <v>491</v>
       </c>
       <c r="E15">
-        <v>3042</v>
+        <v>3268</v>
       </c>
       <c r="F15">
-        <v>194</v>
+        <v>246</v>
       </c>
       <c r="G15">
-        <v>1522</v>
+        <v>1636</v>
       </c>
       <c r="H15">
-        <v>304</v>
+        <v>327</v>
       </c>
       <c r="I15">
-        <v>1511</v>
+        <v>1590</v>
       </c>
       <c r="J15">
-        <v>10628</v>
+        <v>10749</v>
       </c>
     </row>
     <row r="16">
@@ -694,31 +706,31 @@
         </is>
       </c>
       <c r="B16">
-        <v>7630</v>
+        <v>7843</v>
       </c>
       <c r="C16">
         <v>1.05</v>
       </c>
       <c r="D16">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="E16">
-        <v>3165</v>
+        <v>3403</v>
       </c>
       <c r="F16">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="G16">
-        <v>1583</v>
+        <v>1703</v>
       </c>
       <c r="H16">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="I16">
-        <v>1612</v>
+        <v>1695</v>
       </c>
       <c r="J16">
-        <v>12241</v>
+        <v>12444</v>
       </c>
     </row>
     <row r="17">
@@ -728,31 +740,31 @@
         </is>
       </c>
       <c r="B17">
-        <v>8011</v>
+        <v>8236</v>
       </c>
       <c r="C17">
         <v>1.05</v>
       </c>
       <c r="D17">
-        <v>427</v>
+        <v>439</v>
       </c>
       <c r="E17">
-        <v>3285</v>
+        <v>3535</v>
       </c>
       <c r="F17">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="G17">
-        <v>1644</v>
+        <v>1770</v>
       </c>
       <c r="H17">
-        <v>329</v>
+        <v>354</v>
       </c>
       <c r="I17">
-        <v>1718</v>
+        <v>1805</v>
       </c>
       <c r="J17">
-        <v>13959</v>
+        <v>14249</v>
       </c>
     </row>
     <row r="18">
@@ -762,31 +774,31 @@
         </is>
       </c>
       <c r="B18">
-        <v>8412</v>
+        <v>8647</v>
       </c>
       <c r="C18">
         <v>1.05</v>
       </c>
       <c r="D18">
-        <v>448</v>
+        <v>461</v>
       </c>
       <c r="E18">
-        <v>3473</v>
+        <v>3675</v>
       </c>
       <c r="F18">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="G18">
-        <v>1738</v>
+        <v>1839</v>
       </c>
       <c r="H18">
-        <v>348</v>
+        <v>368</v>
       </c>
       <c r="I18">
-        <v>1820</v>
+        <v>1911</v>
       </c>
       <c r="J18">
-        <v>15779</v>
+        <v>16160</v>
       </c>
     </row>
     <row r="19">
@@ -796,31 +808,31 @@
         </is>
       </c>
       <c r="B19">
-        <v>8833</v>
+        <v>9080</v>
       </c>
       <c r="C19">
         <v>1.05</v>
       </c>
       <c r="D19">
-        <v>470</v>
+        <v>484</v>
       </c>
       <c r="E19">
-        <v>3675</v>
+        <v>3839</v>
       </c>
       <c r="F19">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="G19">
-        <v>1838</v>
+        <v>1920</v>
       </c>
       <c r="H19">
-        <v>368</v>
+        <v>384</v>
       </c>
       <c r="I19">
-        <v>1930</v>
+        <v>2026</v>
       </c>
       <c r="J19">
-        <v>17710</v>
+        <v>18187</v>
       </c>
     </row>
     <row r="20">
@@ -830,31 +842,31 @@
         </is>
       </c>
       <c r="B20">
-        <v>9274</v>
+        <v>9534</v>
       </c>
       <c r="C20">
         <v>1.05</v>
       </c>
       <c r="D20">
-        <v>494</v>
+        <v>508</v>
       </c>
       <c r="E20">
-        <v>3875</v>
+        <v>4047</v>
       </c>
       <c r="F20">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="G20">
-        <v>1939</v>
+        <v>2025</v>
       </c>
       <c r="H20">
-        <v>388</v>
+        <v>405</v>
       </c>
       <c r="I20">
-        <v>2038</v>
+        <v>2139</v>
       </c>
       <c r="J20">
-        <v>19748</v>
+        <v>20326</v>
       </c>
     </row>
     <row r="21">
@@ -864,31 +876,31 @@
         </is>
       </c>
       <c r="B21">
-        <v>9738</v>
+        <v>10010</v>
       </c>
       <c r="C21">
         <v>1.05</v>
       </c>
       <c r="D21">
-        <v>519</v>
+        <v>533</v>
       </c>
       <c r="E21">
-        <v>4083</v>
+        <v>4263</v>
       </c>
       <c r="F21">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="G21">
-        <v>2043</v>
+        <v>2132</v>
       </c>
       <c r="H21">
-        <v>409</v>
+        <v>426</v>
       </c>
       <c r="I21">
-        <v>2150</v>
+        <v>2255</v>
       </c>
       <c r="J21">
-        <v>21898</v>
+        <v>22580</v>
       </c>
     </row>
   </sheetData>
@@ -1028,19 +1040,19 @@
         </is>
       </c>
       <c r="C5">
-        <v>8011</v>
+        <v>8236</v>
       </c>
       <c r="D5">
-        <v>1644</v>
+        <v>1770</v>
       </c>
       <c r="E5">
-        <v>329</v>
+        <v>354</v>
       </c>
       <c r="F5">
-        <v>6252</v>
+        <v>6542</v>
       </c>
       <c r="G5">
-        <v>13959</v>
+        <v>14249</v>
       </c>
     </row>
     <row r="6">
@@ -1055,19 +1067,19 @@
         </is>
       </c>
       <c r="C6">
-        <v>9738</v>
+        <v>10010</v>
       </c>
       <c r="D6">
-        <v>2043</v>
+        <v>2132</v>
       </c>
       <c r="E6">
-        <v>409</v>
+        <v>426</v>
       </c>
       <c r="F6">
-        <v>7939</v>
+        <v>8331</v>
       </c>
       <c r="G6">
-        <v>21898</v>
+        <v>22580</v>
       </c>
     </row>
   </sheetData>
@@ -1546,31 +1558,31 @@
         </is>
       </c>
       <c r="B14">
-        <v>6921</v>
+        <v>7030</v>
       </c>
       <c r="C14">
-        <v>1.05</v>
+        <v>1.067</v>
       </c>
       <c r="D14">
-        <v>369</v>
+        <v>491</v>
       </c>
       <c r="E14">
-        <v>2891</v>
+        <v>3013</v>
       </c>
       <c r="F14">
-        <v>184</v>
+        <v>246</v>
       </c>
       <c r="G14">
-        <v>1446</v>
+        <v>1508</v>
       </c>
       <c r="H14">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="I14">
-        <v>1605</v>
+        <v>1662</v>
       </c>
       <c r="J14">
-        <v>10849</v>
+        <v>10906</v>
       </c>
     </row>
     <row r="15">
@@ -1580,31 +1592,31 @@
         </is>
       </c>
       <c r="B15">
-        <v>7267</v>
+        <v>7470</v>
       </c>
       <c r="C15">
-        <v>1.05</v>
+        <v>1.062</v>
       </c>
       <c r="D15">
-        <v>387</v>
+        <v>491</v>
       </c>
       <c r="E15">
-        <v>3042</v>
+        <v>3268</v>
       </c>
       <c r="F15">
-        <v>194</v>
+        <v>246</v>
       </c>
       <c r="G15">
-        <v>1522</v>
+        <v>1636</v>
       </c>
       <c r="H15">
-        <v>304</v>
+        <v>327</v>
       </c>
       <c r="I15">
-        <v>1708</v>
+        <v>1812</v>
       </c>
       <c r="J15">
-        <v>12557</v>
+        <v>12718</v>
       </c>
     </row>
     <row r="16">
@@ -1614,31 +1626,31 @@
         </is>
       </c>
       <c r="B16">
-        <v>7630</v>
+        <v>7843</v>
       </c>
       <c r="C16">
         <v>1.05</v>
       </c>
       <c r="D16">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="E16">
-        <v>3165</v>
+        <v>3403</v>
       </c>
       <c r="F16">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="G16">
-        <v>1583</v>
+        <v>1703</v>
       </c>
       <c r="H16">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="I16">
-        <v>1803</v>
+        <v>1914</v>
       </c>
       <c r="J16">
-        <v>14360</v>
+        <v>14632</v>
       </c>
     </row>
     <row r="17">
@@ -1648,31 +1660,31 @@
         </is>
       </c>
       <c r="B17">
-        <v>8011</v>
+        <v>8236</v>
       </c>
       <c r="C17">
         <v>1.05</v>
       </c>
       <c r="D17">
-        <v>427</v>
+        <v>439</v>
       </c>
       <c r="E17">
-        <v>3285</v>
+        <v>3535</v>
       </c>
       <c r="F17">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="G17">
-        <v>1644</v>
+        <v>1770</v>
       </c>
       <c r="H17">
-        <v>329</v>
+        <v>354</v>
       </c>
       <c r="I17">
-        <v>1901</v>
+        <v>2017</v>
       </c>
       <c r="J17">
-        <v>16262</v>
+        <v>16649</v>
       </c>
     </row>
     <row r="18">
@@ -1682,31 +1694,31 @@
         </is>
       </c>
       <c r="B18">
-        <v>8412</v>
+        <v>8647</v>
       </c>
       <c r="C18">
         <v>1.05</v>
       </c>
       <c r="D18">
-        <v>448</v>
+        <v>461</v>
       </c>
       <c r="E18">
-        <v>3473</v>
+        <v>3675</v>
       </c>
       <c r="F18">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="G18">
-        <v>1738</v>
+        <v>1839</v>
       </c>
       <c r="H18">
-        <v>348</v>
+        <v>368</v>
       </c>
       <c r="I18">
-        <v>2013</v>
+        <v>2120</v>
       </c>
       <c r="J18">
-        <v>18275</v>
+        <v>18769</v>
       </c>
     </row>
     <row r="19">
@@ -1716,31 +1728,31 @@
         </is>
       </c>
       <c r="B19">
-        <v>8833</v>
+        <v>9080</v>
       </c>
       <c r="C19">
         <v>1.05</v>
       </c>
       <c r="D19">
-        <v>470</v>
+        <v>484</v>
       </c>
       <c r="E19">
-        <v>3675</v>
+        <v>3839</v>
       </c>
       <c r="F19">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="G19">
-        <v>1838</v>
+        <v>1920</v>
       </c>
       <c r="H19">
-        <v>368</v>
+        <v>384</v>
       </c>
       <c r="I19">
-        <v>2133</v>
+        <v>2234</v>
       </c>
       <c r="J19">
-        <v>20407</v>
+        <v>21003</v>
       </c>
     </row>
     <row r="20">
@@ -1750,31 +1762,31 @@
         </is>
       </c>
       <c r="B20">
-        <v>9274</v>
+        <v>9534</v>
       </c>
       <c r="C20">
         <v>1.05</v>
       </c>
       <c r="D20">
-        <v>494</v>
+        <v>508</v>
       </c>
       <c r="E20">
-        <v>3875</v>
+        <v>4047</v>
       </c>
       <c r="F20">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="G20">
-        <v>1939</v>
+        <v>2025</v>
       </c>
       <c r="H20">
-        <v>388</v>
+        <v>405</v>
       </c>
       <c r="I20">
-        <v>2251</v>
+        <v>2357</v>
       </c>
       <c r="J20">
-        <v>22658</v>
+        <v>23361</v>
       </c>
     </row>
     <row r="21">
@@ -1784,31 +1796,31 @@
         </is>
       </c>
       <c r="B21">
-        <v>9738</v>
+        <v>10010</v>
       </c>
       <c r="C21">
         <v>1.05</v>
       </c>
       <c r="D21">
-        <v>519</v>
+        <v>533</v>
       </c>
       <c r="E21">
-        <v>4083</v>
+        <v>4263</v>
       </c>
       <c r="F21">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="G21">
-        <v>2043</v>
+        <v>2132</v>
       </c>
       <c r="H21">
-        <v>409</v>
+        <v>426</v>
       </c>
       <c r="I21">
-        <v>2373</v>
+        <v>2484</v>
       </c>
       <c r="J21">
-        <v>25031</v>
+        <v>25844</v>
       </c>
     </row>
   </sheetData>
@@ -1948,19 +1960,19 @@
         </is>
       </c>
       <c r="C5">
-        <v>8011</v>
+        <v>8236</v>
       </c>
       <c r="D5">
-        <v>1644</v>
+        <v>1770</v>
       </c>
       <c r="E5">
-        <v>329</v>
+        <v>354</v>
       </c>
       <c r="F5">
-        <v>7017</v>
+        <v>7405</v>
       </c>
       <c r="G5">
-        <v>16262</v>
+        <v>16649</v>
       </c>
     </row>
     <row r="6">
@@ -1975,19 +1987,19 @@
         </is>
       </c>
       <c r="C6">
-        <v>9738</v>
+        <v>10010</v>
       </c>
       <c r="D6">
-        <v>2043</v>
+        <v>2132</v>
       </c>
       <c r="E6">
-        <v>409</v>
+        <v>426</v>
       </c>
       <c r="F6">
-        <v>8769</v>
+        <v>9195</v>
       </c>
       <c r="G6">
-        <v>25031</v>
+        <v>25844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: refine sbcs revenue notation
</commit_message>
<xml_diff>
--- a/deck-system/decks/umee-sbcs-kintone-plan-3980/exports/umee-kintonepack-5yr-revenue-plan.xlsx
+++ b/deck-system/decks/umee-sbcs-kintone-plan-3980/exports/umee-kintonepack-5yr-revenue-plan.xlsx
@@ -69,94 +69,106 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>追加提示値</t>
+          <t>金額単位</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FY29Q3は70,304、FY29Q4は74,698を反映</t>
+          <t>千円</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5か年延長</t>
+          <t>追加提示値</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FY30Q1以降、Umee全体売上計画は四半期ごとに1.05倍成長として延長</t>
+          <t>FY29Q3は70,304千円、FY29Q4は74,698千円を反映</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SBC&amp;S取扱見込</t>
+          <t>5か年延長</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Umee Tier3計画IDの50%</t>
+          <t>FY30Q1以降、Umee全体売上計画は四半期ごとに1.05倍成長として延長</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>契約法人</t>
+          <t>SBC&amp;S取扱見込</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SBC&amp;S積上ID ÷ 5ID/法人</t>
+          <t>Umee Tier3計画IDの50%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>継続率</t>
+          <t>契約法人</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>契約開始1年後50%、以降1年ごとに80%</t>
+          <t>SBC&amp;S積上ID ÷ 5ID/法人</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>貴社支払いレベニュー額</t>
+          <t>継続率</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kintone Pack販売価格 ÷ 1.3 × 稼働SBC&amp;S ID × 3ヶ月</t>
+          <t>契約開始1年後50%、以降1年ごとに80%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>価格パターン</t>
+          <t>貴社支払いレベニュー額</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>初年度2,980円または3,980円 / ID / 月、2年目以降5,980円 / ID / 月</t>
+          <t>Kintone Pack販売価格 ÷ 1.3 × 稼働SBC&amp;S ID × 3ヶ月。貴社から再販時の販促費等は加味せず</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>価格パターン</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>初年度2,980円または3,980円 / ID / 月、2年目以降5,980円 / ID / 月</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>FrontAX</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>本試算には含めない</t>
         </is>
@@ -177,7 +189,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Umee全体売上計画(万円)</t>
+          <t>Umee全体売上計画(千円)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -212,12 +224,12 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>貴社支払いレベニュー額(万円)</t>
+          <t>貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>累計貴社支払いレベニュー額(万円)</t>
+          <t>累計貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
     </row>
@@ -228,7 +240,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>3200</v>
+        <v>32000</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -251,10 +263,10 @@
         <v>22</v>
       </c>
       <c r="I2">
-        <v>77</v>
+        <v>770</v>
       </c>
       <c r="J2">
-        <v>77</v>
+        <v>770</v>
       </c>
     </row>
     <row r="3">
@@ -264,7 +276,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>3400</v>
+        <v>34000</v>
       </c>
       <c r="C3">
         <v>1.062</v>
@@ -285,10 +297,10 @@
         <v>45</v>
       </c>
       <c r="I3">
-        <v>154</v>
+        <v>1540</v>
       </c>
       <c r="J3">
-        <v>231</v>
+        <v>2311</v>
       </c>
     </row>
     <row r="4">
@@ -298,7 +310,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>3640</v>
+        <v>36400</v>
       </c>
       <c r="C4">
         <v>1.071</v>
@@ -319,10 +331,10 @@
         <v>72</v>
       </c>
       <c r="I4">
-        <v>246</v>
+        <v>2462</v>
       </c>
       <c r="J4">
-        <v>477</v>
+        <v>4773</v>
       </c>
     </row>
     <row r="5">
@@ -332,7 +344,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>3900</v>
+        <v>39000</v>
       </c>
       <c r="C5">
         <v>1.071</v>
@@ -353,10 +365,10 @@
         <v>101</v>
       </c>
       <c r="I5">
-        <v>347</v>
+        <v>3466</v>
       </c>
       <c r="J5">
-        <v>824</v>
+        <v>8239</v>
       </c>
     </row>
     <row r="6">
@@ -366,7 +378,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>4160</v>
+        <v>41600</v>
       </c>
       <c r="C6">
         <v>1.067</v>
@@ -387,10 +399,10 @@
         <v>119</v>
       </c>
       <c r="I6">
-        <v>447</v>
+        <v>4473</v>
       </c>
       <c r="J6">
-        <v>1271</v>
+        <v>12711</v>
       </c>
     </row>
     <row r="7">
@@ -400,7 +412,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>4420</v>
+        <v>44200</v>
       </c>
       <c r="C7">
         <v>1.062</v>
@@ -421,10 +433,10 @@
         <v>137</v>
       </c>
       <c r="I7">
-        <v>548</v>
+        <v>5479</v>
       </c>
       <c r="J7">
-        <v>1819</v>
+        <v>18190</v>
       </c>
     </row>
     <row r="8">
@@ -434,7 +446,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>4732</v>
+        <v>47320</v>
       </c>
       <c r="C8">
         <v>1.071</v>
@@ -455,10 +467,10 @@
         <v>158</v>
       </c>
       <c r="I8">
-        <v>668</v>
+        <v>6679</v>
       </c>
       <c r="J8">
-        <v>2487</v>
+        <v>24869</v>
       </c>
     </row>
     <row r="9">
@@ -468,7 +480,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>5070</v>
+        <v>50700</v>
       </c>
       <c r="C9">
         <v>1.071</v>
@@ -489,10 +501,10 @@
         <v>181</v>
       </c>
       <c r="I9">
-        <v>798</v>
+        <v>7982</v>
       </c>
       <c r="J9">
-        <v>3285</v>
+        <v>32851</v>
       </c>
     </row>
     <row r="10">
@@ -502,7 +514,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>5408</v>
+        <v>54080</v>
       </c>
       <c r="C10">
         <v>1.067</v>
@@ -523,10 +535,10 @@
         <v>202</v>
       </c>
       <c r="I10">
-        <v>913</v>
+        <v>9131</v>
       </c>
       <c r="J10">
-        <v>4198</v>
+        <v>41982</v>
       </c>
     </row>
     <row r="11">
@@ -536,7 +548,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>5746</v>
+        <v>57460</v>
       </c>
       <c r="C11">
         <v>1.062</v>
@@ -557,10 +569,10 @@
         <v>223</v>
       </c>
       <c r="I11">
-        <v>1028</v>
+        <v>10279</v>
       </c>
       <c r="J11">
-        <v>5226</v>
+        <v>52261</v>
       </c>
     </row>
     <row r="12">
@@ -570,7 +582,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>6152</v>
+        <v>61516</v>
       </c>
       <c r="C12">
         <v>1.071</v>
@@ -591,10 +603,10 @@
         <v>249</v>
       </c>
       <c r="I12">
-        <v>1166</v>
+        <v>11659</v>
       </c>
       <c r="J12">
-        <v>6392</v>
+        <v>63920</v>
       </c>
     </row>
     <row r="13">
@@ -604,7 +616,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>6591</v>
+        <v>65910</v>
       </c>
       <c r="C13">
         <v>1.071</v>
@@ -625,10 +637,10 @@
         <v>276</v>
       </c>
       <c r="I13">
-        <v>1315</v>
+        <v>13154</v>
       </c>
       <c r="J13">
-        <v>7707</v>
+        <v>77074</v>
       </c>
     </row>
     <row r="14">
@@ -638,7 +650,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>7030</v>
+        <v>70304</v>
       </c>
       <c r="C14">
         <v>1.067</v>
@@ -659,10 +671,10 @@
         <v>302</v>
       </c>
       <c r="I14">
-        <v>1452</v>
+        <v>14525</v>
       </c>
       <c r="J14">
-        <v>9160</v>
+        <v>91599</v>
       </c>
     </row>
     <row r="15">
@@ -672,7 +684,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>7470</v>
+        <v>74698</v>
       </c>
       <c r="C15">
         <v>1.062</v>
@@ -693,10 +705,10 @@
         <v>327</v>
       </c>
       <c r="I15">
-        <v>1590</v>
+        <v>15896</v>
       </c>
       <c r="J15">
-        <v>10749</v>
+        <v>107494</v>
       </c>
     </row>
     <row r="16">
@@ -706,7 +718,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>7843</v>
+        <v>78433</v>
       </c>
       <c r="C16">
         <v>1.05</v>
@@ -727,10 +739,10 @@
         <v>341</v>
       </c>
       <c r="I16">
-        <v>1695</v>
+        <v>16950</v>
       </c>
       <c r="J16">
-        <v>12444</v>
+        <v>124445</v>
       </c>
     </row>
     <row r="17">
@@ -740,7 +752,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>8236</v>
+        <v>82355</v>
       </c>
       <c r="C17">
         <v>1.05</v>
@@ -761,10 +773,10 @@
         <v>354</v>
       </c>
       <c r="I17">
-        <v>1805</v>
+        <v>18047</v>
       </c>
       <c r="J17">
-        <v>14249</v>
+        <v>142491</v>
       </c>
     </row>
     <row r="18">
@@ -774,7 +786,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>8647</v>
+        <v>86473</v>
       </c>
       <c r="C18">
         <v>1.05</v>
@@ -795,10 +807,10 @@
         <v>368</v>
       </c>
       <c r="I18">
-        <v>1911</v>
+        <v>19113</v>
       </c>
       <c r="J18">
-        <v>16160</v>
+        <v>161605</v>
       </c>
     </row>
     <row r="19">
@@ -808,7 +820,7 @@
         </is>
       </c>
       <c r="B19">
-        <v>9080</v>
+        <v>90797</v>
       </c>
       <c r="C19">
         <v>1.05</v>
@@ -829,10 +841,10 @@
         <v>384</v>
       </c>
       <c r="I19">
-        <v>2026</v>
+        <v>20262</v>
       </c>
       <c r="J19">
-        <v>18187</v>
+        <v>181867</v>
       </c>
     </row>
     <row r="20">
@@ -842,7 +854,7 @@
         </is>
       </c>
       <c r="B20">
-        <v>9534</v>
+        <v>95337</v>
       </c>
       <c r="C20">
         <v>1.05</v>
@@ -863,10 +875,10 @@
         <v>405</v>
       </c>
       <c r="I20">
-        <v>2139</v>
+        <v>21390</v>
       </c>
       <c r="J20">
-        <v>20326</v>
+        <v>203257</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +888,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>10010</v>
+        <v>100104</v>
       </c>
       <c r="C21">
         <v>1.05</v>
@@ -897,10 +909,10 @@
         <v>426</v>
       </c>
       <c r="I21">
-        <v>2255</v>
+        <v>22547</v>
       </c>
       <c r="J21">
-        <v>22580</v>
+        <v>225804</v>
       </c>
     </row>
   </sheetData>
@@ -923,7 +935,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>年度末Umee全体売上計画(万円)</t>
+          <t>年度末Umee全体売上計画(千円)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -938,12 +950,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>年度貴社支払いレベニュー額(万円)</t>
+          <t>年度貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>累計貴社支払いレベニュー額(万円)</t>
+          <t>累計貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
     </row>
@@ -959,7 +971,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>3900</v>
+        <v>39000</v>
       </c>
       <c r="D2">
         <v>504</v>
@@ -968,10 +980,10 @@
         <v>101</v>
       </c>
       <c r="F2">
-        <v>824</v>
+        <v>8239</v>
       </c>
       <c r="G2">
-        <v>824</v>
+        <v>8239</v>
       </c>
     </row>
     <row r="3">
@@ -986,7 +998,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>5070</v>
+        <v>50700</v>
       </c>
       <c r="D3">
         <v>907</v>
@@ -995,10 +1007,10 @@
         <v>181</v>
       </c>
       <c r="F3">
-        <v>2461</v>
+        <v>24613</v>
       </c>
       <c r="G3">
-        <v>3285</v>
+        <v>32851</v>
       </c>
     </row>
     <row r="4">
@@ -1013,7 +1025,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>6591</v>
+        <v>65910</v>
       </c>
       <c r="D4">
         <v>1380</v>
@@ -1022,10 +1034,10 @@
         <v>276</v>
       </c>
       <c r="F4">
-        <v>4422</v>
+        <v>44223</v>
       </c>
       <c r="G4">
-        <v>7707</v>
+        <v>77074</v>
       </c>
     </row>
     <row r="5">
@@ -1040,7 +1052,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>8236</v>
+        <v>82355</v>
       </c>
       <c r="D5">
         <v>1770</v>
@@ -1049,10 +1061,10 @@
         <v>354</v>
       </c>
       <c r="F5">
-        <v>6542</v>
+        <v>65418</v>
       </c>
       <c r="G5">
-        <v>14249</v>
+        <v>142491</v>
       </c>
     </row>
     <row r="6">
@@ -1067,7 +1079,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>10010</v>
+        <v>100104</v>
       </c>
       <c r="D6">
         <v>2132</v>
@@ -1076,10 +1088,10 @@
         <v>426</v>
       </c>
       <c r="F6">
-        <v>8331</v>
+        <v>83313</v>
       </c>
       <c r="G6">
-        <v>22580</v>
+        <v>225804</v>
       </c>
     </row>
   </sheetData>
@@ -1097,7 +1109,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Umee全体売上計画(万円)</t>
+          <t>Umee全体売上計画(千円)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1132,12 +1144,12 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>貴社支払いレベニュー額(万円)</t>
+          <t>貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>累計貴社支払いレベニュー額(万円)</t>
+          <t>累計貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1160,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>3200</v>
+        <v>32000</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1171,10 +1183,10 @@
         <v>22</v>
       </c>
       <c r="I2">
-        <v>103</v>
+        <v>1029</v>
       </c>
       <c r="J2">
-        <v>103</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="3">
@@ -1184,7 +1196,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>3400</v>
+        <v>34000</v>
       </c>
       <c r="C3">
         <v>1.062</v>
@@ -1205,10 +1217,10 @@
         <v>45</v>
       </c>
       <c r="I3">
-        <v>206</v>
+        <v>2057</v>
       </c>
       <c r="J3">
-        <v>309</v>
+        <v>3086</v>
       </c>
     </row>
     <row r="4">
@@ -1218,7 +1230,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>3640</v>
+        <v>36400</v>
       </c>
       <c r="C4">
         <v>1.071</v>
@@ -1239,10 +1251,10 @@
         <v>72</v>
       </c>
       <c r="I4">
-        <v>329</v>
+        <v>3288</v>
       </c>
       <c r="J4">
-        <v>637</v>
+        <v>6374</v>
       </c>
     </row>
     <row r="5">
@@ -1252,7 +1264,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>3900</v>
+        <v>39000</v>
       </c>
       <c r="C5">
         <v>1.071</v>
@@ -1273,10 +1285,10 @@
         <v>101</v>
       </c>
       <c r="I5">
-        <v>463</v>
+        <v>4629</v>
       </c>
       <c r="J5">
-        <v>1100</v>
+        <v>11003</v>
       </c>
     </row>
     <row r="6">
@@ -1286,7 +1298,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>4160</v>
+        <v>41600</v>
       </c>
       <c r="C6">
         <v>1.067</v>
@@ -1307,10 +1319,10 @@
         <v>119</v>
       </c>
       <c r="I6">
-        <v>571</v>
+        <v>5714</v>
       </c>
       <c r="J6">
-        <v>1672</v>
+        <v>16717</v>
       </c>
     </row>
     <row r="7">
@@ -1320,7 +1332,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>4420</v>
+        <v>44200</v>
       </c>
       <c r="C7">
         <v>1.062</v>
@@ -1341,10 +1353,10 @@
         <v>137</v>
       </c>
       <c r="I7">
-        <v>680</v>
+        <v>6799</v>
       </c>
       <c r="J7">
-        <v>2352</v>
+        <v>23516</v>
       </c>
     </row>
     <row r="8">
@@ -1354,7 +1366,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>4732</v>
+        <v>47320</v>
       </c>
       <c r="C8">
         <v>1.071</v>
@@ -1375,10 +1387,10 @@
         <v>158</v>
       </c>
       <c r="I8">
-        <v>809</v>
+        <v>8091</v>
       </c>
       <c r="J8">
-        <v>3161</v>
+        <v>31608</v>
       </c>
     </row>
     <row r="9">
@@ -1388,7 +1400,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>5070</v>
+        <v>50700</v>
       </c>
       <c r="C9">
         <v>1.071</v>
@@ -1409,10 +1421,10 @@
         <v>181</v>
       </c>
       <c r="I9">
-        <v>949</v>
+        <v>9494</v>
       </c>
       <c r="J9">
-        <v>4110</v>
+        <v>41101</v>
       </c>
     </row>
     <row r="10">
@@ -1422,7 +1434,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>5408</v>
+        <v>54080</v>
       </c>
       <c r="C10">
         <v>1.067</v>
@@ -1443,10 +1455,10 @@
         <v>202</v>
       </c>
       <c r="I10">
-        <v>1074</v>
+        <v>10741</v>
       </c>
       <c r="J10">
-        <v>5184</v>
+        <v>51843</v>
       </c>
     </row>
     <row r="11">
@@ -1456,7 +1468,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>5746</v>
+        <v>57460</v>
       </c>
       <c r="C11">
         <v>1.062</v>
@@ -1477,10 +1489,10 @@
         <v>223</v>
       </c>
       <c r="I11">
-        <v>1199</v>
+        <v>11989</v>
       </c>
       <c r="J11">
-        <v>6383</v>
+        <v>63832</v>
       </c>
     </row>
     <row r="12">
@@ -1490,7 +1502,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>6152</v>
+        <v>61516</v>
       </c>
       <c r="C12">
         <v>1.071</v>
@@ -1511,10 +1523,10 @@
         <v>249</v>
       </c>
       <c r="I12">
-        <v>1349</v>
+        <v>13492</v>
       </c>
       <c r="J12">
-        <v>7732</v>
+        <v>77323</v>
       </c>
     </row>
     <row r="13">
@@ -1524,7 +1536,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>6591</v>
+        <v>65910</v>
       </c>
       <c r="C13">
         <v>1.071</v>
@@ -1545,10 +1557,10 @@
         <v>276</v>
       </c>
       <c r="I13">
-        <v>1512</v>
+        <v>15118</v>
       </c>
       <c r="J13">
-        <v>9244</v>
+        <v>92441</v>
       </c>
     </row>
     <row r="14">
@@ -1558,7 +1570,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>7030</v>
+        <v>70304</v>
       </c>
       <c r="C14">
         <v>1.067</v>
@@ -1579,10 +1591,10 @@
         <v>302</v>
       </c>
       <c r="I14">
-        <v>1662</v>
+        <v>16620</v>
       </c>
       <c r="J14">
-        <v>10906</v>
+        <v>109061</v>
       </c>
     </row>
     <row r="15">
@@ -1592,7 +1604,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>7470</v>
+        <v>74698</v>
       </c>
       <c r="C15">
         <v>1.062</v>
@@ -1613,10 +1625,10 @@
         <v>327</v>
       </c>
       <c r="I15">
-        <v>1812</v>
+        <v>18123</v>
       </c>
       <c r="J15">
-        <v>12718</v>
+        <v>127184</v>
       </c>
     </row>
     <row r="16">
@@ -1626,7 +1638,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>7843</v>
+        <v>78433</v>
       </c>
       <c r="C16">
         <v>1.05</v>
@@ -1647,10 +1659,10 @@
         <v>341</v>
       </c>
       <c r="I16">
-        <v>1914</v>
+        <v>19136</v>
       </c>
       <c r="J16">
-        <v>14632</v>
+        <v>146319</v>
       </c>
     </row>
     <row r="17">
@@ -1660,7 +1672,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>8236</v>
+        <v>82355</v>
       </c>
       <c r="C17">
         <v>1.05</v>
@@ -1681,10 +1693,10 @@
         <v>354</v>
       </c>
       <c r="I17">
-        <v>2017</v>
+        <v>20172</v>
       </c>
       <c r="J17">
-        <v>16649</v>
+        <v>166491</v>
       </c>
     </row>
     <row r="18">
@@ -1694,7 +1706,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>8647</v>
+        <v>86473</v>
       </c>
       <c r="C18">
         <v>1.05</v>
@@ -1715,10 +1727,10 @@
         <v>368</v>
       </c>
       <c r="I18">
-        <v>2120</v>
+        <v>21202</v>
       </c>
       <c r="J18">
-        <v>18769</v>
+        <v>187693</v>
       </c>
     </row>
     <row r="19">
@@ -1728,7 +1740,7 @@
         </is>
       </c>
       <c r="B19">
-        <v>9080</v>
+        <v>90797</v>
       </c>
       <c r="C19">
         <v>1.05</v>
@@ -1749,10 +1761,10 @@
         <v>384</v>
       </c>
       <c r="I19">
-        <v>2234</v>
+        <v>22341</v>
       </c>
       <c r="J19">
-        <v>21003</v>
+        <v>210035</v>
       </c>
     </row>
     <row r="20">
@@ -1762,7 +1774,7 @@
         </is>
       </c>
       <c r="B20">
-        <v>9534</v>
+        <v>95337</v>
       </c>
       <c r="C20">
         <v>1.05</v>
@@ -1783,10 +1795,10 @@
         <v>405</v>
       </c>
       <c r="I20">
-        <v>2357</v>
+        <v>23573</v>
       </c>
       <c r="J20">
-        <v>23361</v>
+        <v>233608</v>
       </c>
     </row>
     <row r="21">
@@ -1796,7 +1808,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>10010</v>
+        <v>100104</v>
       </c>
       <c r="C21">
         <v>1.05</v>
@@ -1817,10 +1829,10 @@
         <v>426</v>
       </c>
       <c r="I21">
-        <v>2484</v>
+        <v>24837</v>
       </c>
       <c r="J21">
-        <v>25844</v>
+        <v>258444</v>
       </c>
     </row>
   </sheetData>
@@ -1843,7 +1855,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>年度末Umee全体売上計画(万円)</t>
+          <t>年度末Umee全体売上計画(千円)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -1858,12 +1870,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>年度貴社支払いレベニュー額(万円)</t>
+          <t>年度貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>累計貴社支払いレベニュー額(万円)</t>
+          <t>累計貴社支払いレベニュー額(千円)</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1891,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>3900</v>
+        <v>39000</v>
       </c>
       <c r="D2">
         <v>504</v>
@@ -1888,10 +1900,10 @@
         <v>101</v>
       </c>
       <c r="F2">
-        <v>1100</v>
+        <v>11003</v>
       </c>
       <c r="G2">
-        <v>1100</v>
+        <v>11003</v>
       </c>
     </row>
     <row r="3">
@@ -1906,7 +1918,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>5070</v>
+        <v>50700</v>
       </c>
       <c r="D3">
         <v>907</v>
@@ -1915,10 +1927,10 @@
         <v>181</v>
       </c>
       <c r="F3">
-        <v>3010</v>
+        <v>30098</v>
       </c>
       <c r="G3">
-        <v>4110</v>
+        <v>41101</v>
       </c>
     </row>
     <row r="4">
@@ -1933,7 +1945,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>6591</v>
+        <v>65910</v>
       </c>
       <c r="D4">
         <v>1380</v>
@@ -1942,10 +1954,10 @@
         <v>276</v>
       </c>
       <c r="F4">
-        <v>5134</v>
+        <v>51340</v>
       </c>
       <c r="G4">
-        <v>9244</v>
+        <v>92441</v>
       </c>
     </row>
     <row r="5">
@@ -1960,7 +1972,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>8236</v>
+        <v>82355</v>
       </c>
       <c r="D5">
         <v>1770</v>
@@ -1969,10 +1981,10 @@
         <v>354</v>
       </c>
       <c r="F5">
-        <v>7405</v>
+        <v>74051</v>
       </c>
       <c r="G5">
-        <v>16649</v>
+        <v>166491</v>
       </c>
     </row>
     <row r="6">
@@ -1987,7 +1999,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>10010</v>
+        <v>100104</v>
       </c>
       <c r="D6">
         <v>2132</v>
@@ -1996,10 +2008,10 @@
         <v>426</v>
       </c>
       <c r="F6">
-        <v>9195</v>
+        <v>91953</v>
       </c>
       <c r="G6">
-        <v>25844</v>
+        <v>258444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>